<commit_message>
Release v1.3: version Airtable data, --local sync mode, UI and matching fixes
- Commit data/raw/*.csv and data/haystacked.db to repo so any tagged version
  is fully self-contained and runnable without Airtable credentials
- Add sync_airtable.py --local flag to rebuild DB from committed CSVs
- Show AGV Matching step as pending from upload start (not hidden until late)
- Skip min_aisle_width clarification for floor/conveyor-only tenders (no racks)
- Industry README: VNA always implies rack; VNA does not exclude floor/conveyor
- Add CLAUDE.md with project and command documentation
- Add docs/: architecture, matching-rules, ap0-change-guide, test-report

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Mobile AMR" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Representatives" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Vehicle Types" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Field Fallbacks" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -2614,8 +2615,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B5:F5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -2630,7 +2631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="43" min="1" max="1"/>
@@ -2708,6 +2709,21 @@
           <t>Tender JSON Key</t>
         </is>
       </c>
+      <c r="L2" s="43" t="inlineStr">
+        <is>
+          <t>Scoring Rule</t>
+        </is>
+      </c>
+      <c r="M2" s="43" t="inlineStr">
+        <is>
+          <t>Threshold 1</t>
+        </is>
+      </c>
+      <c r="N2" s="43" t="inlineStr">
+        <is>
+          <t>Threshold 2</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1" s="44">
       <c r="A3" s="72" t="inlineStr">
@@ -2749,7 +2765,7 @@
       </c>
       <c r="G4" s="66" t="inlineStr">
         <is>
-          <t>Navigation technology. Output from allowed values only, comma-separated. null = not stated.</t>
+          <t>Navigation technology used by the AGV. Output from allowed values only, comma-separated. Mapping rules: 'SLAM' / 'natural feature' / 'free navigation' / 'marker-free' / 'environment mapping' / 'contour-based' → 'Natural Feature (SLAM)'; 'laser reflector' / 'reflector marker' / 'laser scanner with reflectors' → 'Laser Reflector'; 'magnetic tape' / 'magnetic stripe' → 'Magnetic Tape'; 'QR code' / 'barcode' / 'data matrix' → 'QR/DM Code'; 'inductive loop' / 'wire guidance' → 'Inductive Loop'; 'vision' / 'camera-based' → 'Vision'. If multiple navigation types are required, list all. null = not stated in the document.</t>
         </is>
       </c>
       <c r="H4" s="73" t="n"/>
@@ -2964,7 +2980,7 @@
       </c>
       <c r="G10" s="66" t="inlineStr">
         <is>
-          <t>Max rated load. Source: spec 'payload / load capacity'. Hard filter vs. the buyer's heaviest unit load. Use rated, not peak.</t>
+          <t>Maximum payload the AGV must carry per trip. CONSERVATIVE RULE (KO_IF_LT): extract the MAXIMUM loaded weight found in the document — the supplier must meet or exceed this. In pallet tables: use 'Max Loaded weight' / 'gross weight' — IGNORE 'tare weight' / 'empty pallet weight'. If multiple load types are listed, report the heaviest. Output in kg. Null if not stated anywhere.</t>
         </is>
       </c>
       <c r="H10" s="73" t="n"/>
@@ -3551,6 +3567,17 @@
       <c r="J25" s="100" t="n">
         <v>5</v>
       </c>
+      <c r="L25" s="43" t="inlineStr">
+        <is>
+          <t>tiered_lower</t>
+        </is>
+      </c>
+      <c r="M25" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="N25" s="43" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="44">
       <c r="A26" s="72" t="inlineStr">
@@ -3637,6 +3664,14 @@
       <c r="J28" s="100" t="n">
         <v>7</v>
       </c>
+      <c r="L28" s="43" t="inlineStr">
+        <is>
+          <t>threshold_upper</t>
+        </is>
+      </c>
+      <c r="M28" s="43" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="29" ht="33.75" customHeight="1" s="44">
       <c r="A29" s="64" t="inlineStr">
@@ -3716,6 +3751,11 @@
       <c r="J30" s="100" t="n">
         <v>6</v>
       </c>
+      <c r="L30" s="43" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="33.75" customHeight="1" s="44">
       <c r="A31" s="64" t="inlineStr">
@@ -3806,6 +3846,11 @@
       <c r="J33" s="100" t="n">
         <v>5</v>
       </c>
+      <c r="L33" s="43" t="inlineStr">
+        <is>
+          <t>nonempty</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="33.75" customHeight="1" s="44">
       <c r="A34" s="67" t="inlineStr">
@@ -3929,7 +3974,7 @@
       <c r="H37" s="73" t="n"/>
       <c r="I37" s="43" t="inlineStr">
         <is>
-          <t>KO_BOOL_REQUIRED</t>
+          <t>KO_SUBSET</t>
         </is>
       </c>
       <c r="K37" s="43" t="inlineStr">
@@ -4024,6 +4069,11 @@
       <c r="K39" s="43" t="inlineStr">
         <is>
           <t>required_vda5050</t>
+        </is>
+      </c>
+      <c r="L39" s="43" t="inlineStr">
+        <is>
+          <t>bool_cond</t>
         </is>
       </c>
     </row>
@@ -4316,6 +4366,14 @@
       <c r="J48" s="100" t="n">
         <v>15</v>
       </c>
+      <c r="L48" s="43" t="inlineStr">
+        <is>
+          <t>proportional</t>
+        </is>
+      </c>
+      <c r="M48" s="43" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="49" ht="33.75" customHeight="1" s="44">
       <c r="A49" s="67" t="inlineStr">
@@ -4352,6 +4410,17 @@
       <c r="H49" s="77" t="n"/>
       <c r="J49" s="100" t="n">
         <v>10</v>
+      </c>
+      <c r="L49" s="43" t="inlineStr">
+        <is>
+          <t>tiered_lower</t>
+        </is>
+      </c>
+      <c r="M49" s="43" t="n">
+        <v>26</v>
+      </c>
+      <c r="N49" s="43" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="50" ht="33.75" customHeight="1" s="44">
@@ -4928,7 +4997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="43" min="1" max="1"/>
@@ -5006,6 +5075,21 @@
           <t>Tender JSON Key</t>
         </is>
       </c>
+      <c r="L2" s="43" t="inlineStr">
+        <is>
+          <t>Scoring Rule</t>
+        </is>
+      </c>
+      <c r="M2" s="43" t="inlineStr">
+        <is>
+          <t>Threshold 1</t>
+        </is>
+      </c>
+      <c r="N2" s="43" t="inlineStr">
+        <is>
+          <t>Threshold 2</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1" s="44">
       <c r="A3" s="72" t="inlineStr">
@@ -5193,7 +5277,7 @@
       </c>
       <c r="I7" s="43" t="inlineStr">
         <is>
-          <t>KO_IF_LT</t>
+          <t>KO_SUBSET</t>
         </is>
       </c>
       <c r="K7" s="43" t="inlineStr">
@@ -5269,7 +5353,7 @@
       </c>
       <c r="G9" s="69" t="inlineStr">
         <is>
-          <t>Min working aisle in METERS (not mm). Source: 'Gangbreite / aisle width'. If doc states mm (e.g. 2700 mm) → divide by 1000 → 2.7. Hard filter; decisive for VNA.</t>
+          <t>Minimum working aisle width available in the facility, in METERS (not mm). CONSERVATIVE RULE (KO_IF_GT): if multiple aisle widths are stated, extract the MINIMUM — this is the tightest constraint. Example: '2000 mm rack-to-rack, min 1900 mm pallet-to-pallet' → output 1.9. If doc states mm → divide by 1000. Source: 'Gangbreite', 'aisle width', 'corridor width'. Hard filter: decisive for VNA and narrow-aisle forklifts. Null if not stated.</t>
         </is>
       </c>
       <c r="H9" s="77" t="n"/>
@@ -5353,7 +5437,7 @@
       </c>
       <c r="D12" s="81" t="inlineStr">
         <is>
-          <t>K.O.</t>
+          <t>Cond. K.O.</t>
         </is>
       </c>
       <c r="E12" s="76" t="inlineStr">
@@ -5368,7 +5452,7 @@
       </c>
       <c r="G12" s="66" t="inlineStr">
         <is>
-          <t>Forklift drive category. RULE: if required_vna=true → always output 'VNA Turret' (VNA turret trucks are a distinct drive type). Counterbalanced = wide-aisle floor transport (≥3 m), NOT VNA. Output from allowed values only.</t>
+          <t>Forklift drive category. RULE: if required_vna=true → always output 'VNA Turret'. OTHERWISE: ONLY output if the tender document explicitly names the drive type (e.g. 'Gegengewichtsstapler', 'counterbalanced forklift required', 'Schubmaststapler'). DO NOT infer from the task description alone — floor-level pallet transport does NOT imply Counterbalanced; only output if the buyer specifies it. Output from allowed values only, or null.</t>
         </is>
       </c>
       <c r="H12" s="73" t="n"/>
@@ -5429,6 +5513,14 @@
       </c>
       <c r="J14" s="100" t="n">
         <v>8</v>
+      </c>
+      <c r="L14" s="43" t="inlineStr">
+        <is>
+          <t>threshold_lower</t>
+        </is>
+      </c>
+      <c r="M14" s="43" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="15" ht="33.75" customHeight="1" s="44">
@@ -5539,6 +5631,14 @@
       <c r="J17" s="100" t="n">
         <v>6</v>
       </c>
+      <c r="L17" s="43" t="inlineStr">
+        <is>
+          <t>threshold_lower</t>
+        </is>
+      </c>
+      <c r="M17" s="43" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="18" ht="33.75" customHeight="1" s="44">
       <c r="A18" s="64" t="inlineStr">
@@ -5703,6 +5803,11 @@
       <c r="K22" s="43" t="inlineStr">
         <is>
           <t>required_stacking</t>
+        </is>
+      </c>
+      <c r="L22" s="43" t="inlineStr">
+        <is>
+          <t>bool</t>
         </is>
       </c>
     </row>
@@ -6024,7 +6129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="43" min="1" max="1"/>
@@ -6102,6 +6207,21 @@
           <t>Tender JSON Key</t>
         </is>
       </c>
+      <c r="L2" s="43" t="inlineStr">
+        <is>
+          <t>Scoring Rule</t>
+        </is>
+      </c>
+      <c r="M2" s="43" t="inlineStr">
+        <is>
+          <t>Threshold 1</t>
+        </is>
+      </c>
+      <c r="N2" s="43" t="inlineStr">
+        <is>
+          <t>Threshold 2</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1" s="44">
       <c r="A3" s="72" t="inlineStr">
@@ -6300,6 +6420,11 @@
           <t>required_auto_hitch</t>
         </is>
       </c>
+      <c r="L7" s="43" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="33.75" customHeight="1" s="44">
       <c r="A8" s="64" t="inlineStr">
@@ -6499,6 +6624,11 @@
       </c>
       <c r="J13" s="100" t="n">
         <v>6</v>
+      </c>
+      <c r="L13" s="43" t="inlineStr">
+        <is>
+          <t>nonempty</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="44">
@@ -6787,7 +6917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="43" min="1" max="1"/>
@@ -6865,6 +6995,21 @@
           <t>Tender JSON Key</t>
         </is>
       </c>
+      <c r="L2" s="43" t="inlineStr">
+        <is>
+          <t>Scoring Rule</t>
+        </is>
+      </c>
+      <c r="M2" s="43" t="inlineStr">
+        <is>
+          <t>Threshold 1</t>
+        </is>
+      </c>
+      <c r="N2" s="43" t="inlineStr">
+        <is>
+          <t>Threshold 2</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1" s="44">
       <c r="A3" s="72" t="inlineStr">
@@ -7013,6 +7158,11 @@
       <c r="J6" s="100" t="n">
         <v>7</v>
       </c>
+      <c r="L6" s="43" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="33.75" customHeight="1" s="44">
       <c r="A7" s="67" t="inlineStr">
@@ -7872,6 +8022,17 @@
       </c>
       <c r="J31" s="100" t="n">
         <v>8</v>
+      </c>
+      <c r="L31" s="43" t="inlineStr">
+        <is>
+          <t>tiered_upper</t>
+        </is>
+      </c>
+      <c r="M31" s="43" t="n">
+        <v>300</v>
+      </c>
+      <c r="N31" s="43" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="32" ht="33.75" customHeight="1" s="44">
@@ -8897,7 +9058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="44" min="1" max="1"/>
@@ -9076,12 +9237,12 @@
       <c r="E6" s="104" t="inlineStr"/>
       <c r="F6" s="104" t="inlineStr">
         <is>
-          <t>AGV transports pallets on wide aisles (≥3m) or open floor between fixed transfer stations, floor-level pickup/deposit</t>
+          <t>AGV transports pallets on wide aisles (≥3m) or open floor between fixed transfer stations, floor-level pickup/deposit. USE THIS for heavy pallet transport (&gt;1000 kg) in F&amp;B, food production, or manufacturing environments — even when MES or OPC-UA integration is mentioned. The presence of filling lines or MES does NOT imply Mobile AMR if payload is heavy.</t>
         </is>
       </c>
       <c r="G6" s="104" t="inlineStr">
         <is>
-          <t>≥3m aisle, floor transport, transfer stations, warehouse/logistics</t>
+          <t>≥3m aisle, floor transport, transfer stations, warehouse/logistics, heavy pallet (&gt;1000 kg)</t>
         </is>
       </c>
     </row>
@@ -9215,18 +9376,18 @@
       </c>
       <c r="D11" s="104" t="inlineStr">
         <is>
-          <t>amr|mobile robot|fahrroboter|autonomer</t>
+          <t>amr|mobile robot|fahrroboter|autonomer|goods-to-person|goods to person</t>
         </is>
       </c>
       <c r="E11" s="104" t="inlineStr"/>
       <c r="F11" s="104" t="inlineStr">
         <is>
-          <t>Autonomous robot in PRODUCTION or MANUFACTURING environment (filling lines, assembly, processing), or with conveyor/shelf top modules, SLAM navigation, dispatched from MES/WMS. Payload typically &lt;1500 kg.</t>
+          <t>Autonomous robot in PRODUCTION or MANUFACTURING environment (filling lines, assembly, processing), or with conveyor/shelf top modules, SLAM navigation, dispatched from MES/WMS. ONLY use for LIGHT payloads (typically &lt;1000 kg). If payload &gt;1000 kg or if the task is heavy pallet transport → use Forklift AGV instead.</t>
         </is>
       </c>
       <c r="G11" s="104" t="inlineStr">
         <is>
-          <t>production, filling lines, manufacturing, SLAM, MES</t>
+          <t>production, filling lines, manufacturing, SLAM, MES — BUT only if payload &lt;1000 kg</t>
         </is>
       </c>
     </row>
@@ -9337,6 +9498,130 @@
       <c r="E15" s="104" t="inlineStr"/>
       <c r="F15" s="104" t="inlineStr"/>
       <c r="G15" s="104" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>AGV</t>
+        </is>
+      </c>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>Forklift AGV</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D16" s="43" t="inlineStr">
+        <is>
+          <t>agv</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="43" t="inlineStr">
+        <is>
+          <t>Text-based fallbacks for fields the LLM reliably misses. generate_all.py reads these into vehicle_types.json → field_text_fallbacks. app.py applies them after LLM extraction when the field is null.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="43" t="inlineStr">
+        <is>
+          <t>Tender Key</t>
+        </is>
+      </c>
+      <c r="B2" s="43" t="inlineStr">
+        <is>
+          <t>Regex (applied to full PDF text)</t>
+        </is>
+      </c>
+      <c r="C2" s="43" t="inlineStr">
+        <is>
+          <t>Fallback Value (AP0 allowed value)</t>
+        </is>
+      </c>
+      <c r="D2" s="43" t="inlineStr">
+        <is>
+          <t>Only If Null</t>
+        </is>
+      </c>
+      <c r="E2" s="43" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="43" t="inlineStr">
+        <is>
+          <t>required_navigation</t>
+        </is>
+      </c>
+      <c r="B3" s="43" t="inlineStr">
+        <is>
+          <t>(?i)\bSLAM\b</t>
+        </is>
+      </c>
+      <c r="C3" s="43" t="inlineStr">
+        <is>
+          <t>Natural Feature (SLAM)</t>
+        </is>
+      </c>
+      <c r="D3" s="43" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E3" s="43" t="inlineStr">
+        <is>
+          <t>SLAM keyword in document → infer SLAM navigation when LLM extraction returns null</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="43" t="inlineStr">
+        <is>
+          <t>required_navigation</t>
+        </is>
+      </c>
+      <c r="B4" s="43" t="inlineStr">
+        <is>
+          <t>(?i)(natural[\s\-]feature|marker[\s\-]free|free[\s\-]navigat)</t>
+        </is>
+      </c>
+      <c r="C4" s="43" t="inlineStr">
+        <is>
+          <t>Natural Feature (SLAM)</t>
+        </is>
+      </c>
+      <c r="D4" s="43" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E4" s="43" t="inlineStr">
+        <is>
+          <t>Natural feature / marker-free / free navigation wording → SLAM</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix hallucinations and drive_type KO; align test pipeline with production
- Add ANTI-HALLUCINATION Rule 9 to build_system_context() — the active AGV
  system prompt; extraction_system.txt is fallback-only when DB unavailable
- Fix test_pipeline.py to use build_system_context() instead of
  extraction_system.txt, matching production LLM environment
- AP0 xlsx: 7 field descriptions hardened with NULL RULE (temp, IP, humidity,
  gradient, floor flatness, VDA5050); drive_type Level→Context, Operator
  cleared, Description expanded with plain-language type explanations
- Remove dead VNA drive_type injection from app.py (drive_type is CONTEXT,
  VNA hard-gated via vna_capable KO_BOOL_EXCLUSIVE)
- Run 9 results: Dragonfly hallucinations suppressed (all 7 fields null),
  4 VNA suppliers score +16; Mama vehicle type misclassification remains open

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -2615,8 +2615,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B5:F5"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -3225,7 +3225,7 @@
       <c r="F17" s="77" t="n"/>
       <c r="G17" s="69" t="inlineStr">
         <is>
-          <t>Lowest rated operating temperature. Source: 'working temperature'. Cond. K.O.: binds only for cold stores/freezers (-25 °C); standard units bottom out near 0–5 °C.</t>
+          <t>Lowest rated operating temperature. Source: 'working temperature' in environment/operating conditions section. Cond. K.O.: binds only for cold stores/freezers (-25 °C); standard units bottom out near 0–5 °C. NULL RULE: ONLY extract from an explicit °C value in a technical specification section. Do NOT confuse with dates (e.g. '25th May', '2022-05-25'), revision numbers, or project metadata — these are never temperatures. If no operating temperature range is stated → null.</t>
         </is>
       </c>
       <c r="H17" s="77" t="n"/>
@@ -3269,7 +3269,7 @@
       <c r="F18" s="73" t="n"/>
       <c r="G18" s="66" t="inlineStr">
         <is>
-          <t>Highest rated operating temperature. Source: 'working temperature'. Cond. K.O.: relevant only for hot production halls.</t>
+          <t>Highest rated operating temperature. Source: 'working temperature' in environment/operating conditions section. Cond. K.O.: relevant only for hot production halls. NULL RULE: ONLY extract from an explicit °C value in a technical specification. Do NOT confuse with dates, year numbers, or version codes. If not stated → null.</t>
         </is>
       </c>
       <c r="H18" s="73" t="n"/>
@@ -3313,7 +3313,7 @@
       <c r="F19" s="77" t="n"/>
       <c r="G19" s="69" t="inlineStr">
         <is>
-          <t>Max rated relative humidity (non-condensing unless stated). Source: environment spec. Cond. K.O.: binds for wet/washdown areas; pair with ingress_protection_rating.</t>
+          <t>Max rated relative humidity (non-condensing unless stated). Source: environment spec — must appear as a % value. Cond. K.O.: binds for wet/washdown areas; pair with ingress_protection_rating. NULL RULE: null unless a humidity percentage is explicitly stated. Do NOT infer from warehouse type, food industry context, or cold-storage environment.</t>
         </is>
       </c>
       <c r="H19" s="77" t="n"/>
@@ -3357,7 +3357,7 @@
       <c r="F20" s="73" t="n"/>
       <c r="G20" s="66" t="inlineStr">
         <is>
-          <t>IP code for dust/water resistance. Source: spec 'IP rating'. Cond. K.O.: IP52+ binds for dust/moisture/washdown (F&amp;B, beverage); standard AMRs ≈ IP20. 'None' = no rating stated.</t>
+          <t>IP code for dust/water resistance. Source: spec 'IP rating' — must be explicitly printed (e.g. 'IP54', 'IP65'). Cond. K.O.: IP52+ binds for dust/moisture/washdown (F&amp;B, beverage); standard AMRs ≈ IP20. 'None' = no rating stated. NULL RULE: null if no IP code is explicitly stated. Warehouse type, AGV type, and storage environment do NOT imply an IP rating — a VNA high-bay warehouse is NOT necessarily IP65.</t>
         </is>
       </c>
       <c r="H20" s="83" t="inlineStr">
@@ -3453,7 +3453,7 @@
       <c r="F22" s="73" t="n"/>
       <c r="G22" s="66" t="inlineStr">
         <is>
-          <t>Max ramp gradient the loaded unit handles. Source: spec 'gradeability'. Cond. K.O.: binds only where the site has ramps/dock inclines. (moved here — applies to all types)</t>
+          <t>Max ramp gradient the loaded unit handles. Source: spec 'gradeability' — must appear as an explicit % value. Cond. K.O.: binds only where the site has ramps/dock inclines. NULL RULE: null unless a slope or gradient percentage is explicitly stated in the document. Do NOT apply typical industry values (e.g. '5%') when the document is silent on gradients.</t>
         </is>
       </c>
       <c r="H22" s="83" t="inlineStr">
@@ -3501,7 +3501,7 @@
       <c r="F23" s="77" t="n"/>
       <c r="G23" s="69" t="inlineStr">
         <is>
-          <t>Floor flatness the system requires for safe operation/high-lift. Source: install requirements. Cond. K.O.: binds when the site floor is below spec → costly grinding. (moved here — applies to all types)</t>
+          <t>Floor flatness the system requires for safe operation/high-lift. Source: install requirements — must name a standard or value. Cond. K.O.: binds when the site floor is below spec → costly grinding. NULL RULE: null unless a floor quality standard (DIN 15185, FM number, FF number, etc.) or explicit flatness value is named. Do NOT infer from VNA or high-bay context.</t>
         </is>
       </c>
       <c r="H23" s="83" t="inlineStr">
@@ -4050,7 +4050,7 @@
       <c r="F39" s="73" t="n"/>
       <c r="G39" s="66" t="inlineStr">
         <is>
-          <t>Supports VDA 5050 (open AGV↔master-control interface standard). Source: 'VDA 5050 ready'. Cond. K.O.: trending to a hard requirement for large EU multi-vendor tenders.</t>
+          <t>Supports VDA 5050 (open AGV↔master-control interface standard). Source: 'VDA 5050 ready' or 'VDA-5050'. Cond. K.O.: trending to a hard requirement for large EU multi-vendor tenders. NULL RULE: null unless the document literally contains 'VDA 5050' or 'VDA-5050'. Do NOT infer from fleet management, MES/WMS integration, or system openness requirements.</t>
         </is>
       </c>
       <c r="H39" s="83" t="inlineStr">
@@ -5437,7 +5437,7 @@
       </c>
       <c r="D12" s="81" t="inlineStr">
         <is>
-          <t>Cond. K.O.</t>
+          <t>Context</t>
         </is>
       </c>
       <c r="E12" s="76" t="inlineStr">
@@ -5452,15 +5452,17 @@
       </c>
       <c r="G12" s="66" t="inlineStr">
         <is>
-          <t>Forklift drive category. RULE: if required_vna=true → always output 'VNA Turret'. OTHERWISE: ONLY output if the tender document explicitly names the drive type (e.g. 'Gegengewichtsstapler', 'counterbalanced forklift required', 'Schubmaststapler'). DO NOT infer from the task description alone — floor-level pallet transport does NOT imply Counterbalanced; only output if the buyer specifies it. Output from allowed values only, or null.</t>
+          <t>Forklift drive category — describes the physical build of the forklift mechanism. There are five types:
+- Counterbalanced (Gegengewichtsstapler): rear counterweight, no front support legs, forks fully exposed. Can pick pallets directly from the floor and mate with closed conveyors. Wide aisles (≥3 m).
+- Reach Truck (Schubmaststapler): forks extend forward between two front legs. Handles racking in medium aisles (2–3 m), lifts up to ~8 m.
+- Straddle Stacker (Spreizenstapler): load sits between the front legs. Narrower aisles and higher lift than a reach truck.
+- Pallet Mover (Niederhubwagen): low-profile, floor-to-floor transport only, no high-lift to racking.
+- VNA Turret (Schmalgangstapler): only the turret rotates, not the chassis. Ultra-narrow aisles (&lt;2 m), high-bay racking up to 17 m. Always wire- or rail-guided in the aisle.
+EXTRACTION RULE: if required_vna=true → always output 'VNA Turret'. Otherwise: ONLY output if the buyer explicitly names a drive type or forklift category in the document (e.g. 'Gegengewichtsstapler', 'counterbalanced forklift', 'Schubmaststapler', 'reach truck required'). DO NOT infer from the task — floor-level pallet transport does NOT imply Counterbalanced. Output null if the buyer does not specify a drive type.</t>
         </is>
       </c>
       <c r="H12" s="73" t="n"/>
-      <c r="I12" s="102" t="inlineStr">
-        <is>
-          <t>KO_SUBSET</t>
-        </is>
-      </c>
+      <c r="I12" s="102" t="n"/>
       <c r="K12" s="43" t="inlineStr">
         <is>
           <t>required_drive_type</t>

</xml_diff>

<commit_message>
i18n: switch all user-facing text to English
AP0 xlsx + fields.json:
- 122/122 UI Hints translated from German to English
- fill_ui_hints.py updated with English strings

app.py:
- All SSE messages and user-facing errors translated
  (upload, extraction, LLM, validation, plausibility, error paths)

templates/index.html:
- Upload zone, progress, buyer card, shortlist labels
- Clarification dialog title/buttons, field selector, error notices

186 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -2596,8 +2596,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="Q4" s="64" t="inlineStr">
         <is>
-          <t>Welche Navigationsart ist vorgesehen oder erlaubt? (z. B. Natural Feature/SLAM, Magnetband, QR-Code)</t>
+          <t>What navigation type is intended or allowed? (e.g. Natural Feature/SLAM, magnetic tape, QR code)</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="Q5" s="64" t="inlineStr">
         <is>
-          <t>Ist die Installation von Infrastruktur akzeptabel? (z. B. Leitdrähte, Reflektoren, QR-Codes)</t>
+          <t>Is installation of infrastructure (guide wires, reflectors, QR codes) acceptable or explicitly not desired?</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="Q6" s="64" t="inlineStr">
         <is>
-          <t>Wird Außenbetrieb benötigt?</t>
+          <t>Is outdoor operation required?</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="Q7" s="64" t="inlineStr">
         <is>
-          <t>Kann das AGV Hindernissen eigenständig ausweichen ohne anzuhalten?</t>
+          <t>Can the AGV autonomously navigate around obstacles?</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="Q8" s="64" t="inlineStr">
         <is>
-          <t>Muss das AGV in alle Richtungen ohne Wenden fahren können (omnidirektional)?</t>
+          <t>Must the AGV be able to move in all directions without turning (omnidirectional)?</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="Q10" s="64" t="inlineStr">
         <is>
-          <t>Wie hoch ist die maximale Nutzlast pro Ladungsträger? Das AGV muss mindestens dieses Gewicht tragen können (kg).</t>
+          <t>What is the maximum load weight per carrier? The AGV must be able to carry at least this weight.</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="Q11" s="64" t="inlineStr">
         <is>
-          <t>Welche Ladungsträgertypen werden transportiert? (z. B. Europalette, Gitterbox, Behälter — alle zutreffenden auswählen)</t>
+          <t>What type of load carriers will be transported? (e.g. Euro pallet, wire mesh box, container)</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="Q12" s="64" t="inlineStr">
         <is>
-          <t>Muss das AGV mehrere Ladungsträger gleichzeitig transportieren können?</t>
+          <t>Must the AGV be able to transport multiple load carriers simultaneously?</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="Q14" s="64" t="inlineStr">
         <is>
-          <t>Wie schnell soll das AGV maximal fahren? (m/s; z. B. 1,5 m/s)</t>
+          <t>What maximum speed should the AGV achieve? (m/s)</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="Q15" s="64" t="inlineStr">
         <is>
-          <t>Wie lang ist das Fahrzeug? (mm; nur zur Information)</t>
+          <t>Vehicle length. (mm; for reference only)</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="Q16" s="64" t="inlineStr">
         <is>
-          <t>Wie breit ist das Fahrzeug? (mm; nur zur Information)</t>
+          <t>Vehicle width. (mm; for reference only)</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="Q17" s="64" t="inlineStr">
         <is>
-          <t>Wie kalt wird es am Betriebsort mindestens? (°C; z. B. –20 °C für Tiefkühlbereich)</t>
+          <t>What is the minimum temperature at the operating site? (°C; e.g. -20°C for cold storage)</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="Q18" s="64" t="inlineStr">
         <is>
-          <t>Wie warm wird es am Betriebsort maximal? (°C; z. B. 30 °C für Produktionshalle)</t>
+          <t>What is the maximum temperature at the operating site? (°C; e.g. 30°C for production hall)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="Q19" s="64" t="inlineStr">
         <is>
-          <t>Wie hoch ist die maximale relative Luftfeuchtigkeit am Betriebsort? (%)</t>
+          <t>What is the maximum relative humidity at the operating site? (%)</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="Q20" s="64" t="inlineStr">
         <is>
-          <t>Welche Schutzklasse (IP-Klasse) ist am Betriebsort erforderlich? (z. B. IP54 für Spritzwasserschutz)</t>
+          <t>What ingress protection rating (IP class) is required at the operating site? (e.g. IP54 for splash water protection)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="Q21" s="64" t="inlineStr">
         <is>
-          <t>Gibt es Reinraumanforderungen am Betriebsort? (ISO-Klasse; nur ausfüllen wenn Reinraum vorhanden)</t>
+          <t>Are there cleanroom requirements at the operating site? (ISO class; only fill in if cleanroom is present)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="Q22" s="64" t="inlineStr">
         <is>
-          <t>Wie steil ist die steilste Fahrstrecke im Betriebsbereich? (% Steigung; z. B. 1,5 für eine 1,5-%-Rampe)</t>
+          <t>How steep is the steepest driving route in the operating area? (% gradient; e.g. 1.5 for a 1.5% ramp)</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="Q23" s="64" t="inlineStr">
         <is>
-          <t>Gibt es besondere Anforderungen an die Bodenqualität oder -ebenheit?</t>
+          <t>Are there special requirements for floor quality or flatness?</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="Q25" s="64" t="inlineStr">
         <is>
-          <t>Wie präzise muss das AGV an Übergabe- oder Aufnahmepunkten positionieren? (mm zulässige Abweichung)</t>
+          <t>How precisely must the AGV position at transfer or pickup points? (mm deviation)</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="Q27" s="64" t="inlineStr">
         <is>
-          <t>Welcher Batterietyp ist bevorzugt oder erforderlich?</t>
+          <t>What battery type is preferred or required?</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="Q28" s="64" t="inlineStr">
         <is>
-          <t>Wie viele Stunden Betriebszeit pro Ladung werden mindestens benötigt? (h)</t>
+          <t>How many hours of operating time per charge are required as a minimum? (h)</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="Q29" s="64" t="inlineStr">
         <is>
-          <t>Wie lange darf ein vollständiger Ladevorgang maximal dauern? (min)</t>
+          <t>What is the maximum acceptable duration of a full charging cycle? (min)</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="Q30" s="64" t="inlineStr">
         <is>
-          <t>Muss das AGV eigenständig zur Ladestation fahren und automatisch laden?</t>
+          <t>Must the AGV autonomously navigate to the charging station and charge itself?</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="Q31" s="64" t="inlineStr">
         <is>
-          <t>Ist ein schneller manueller Akkuwechsel statt Laden gewünscht?</t>
+          <t>Is fast manual battery swapping desired instead of charging?</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="Q33" s="64" t="inlineStr">
         <is>
-          <t>Welche Sicherheitsnormen müssen erfüllt sein? (z. B. EN ISO 3691-4)</t>
+          <t>Which safety standards must be met? (e.g. EN ISO 3691-4)</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -4029,7 +4029,7 @@
       </c>
       <c r="Q34" s="64" t="inlineStr">
         <is>
-          <t>Welches funktionale Sicherheitsniveau ist gefordert? (z. B. PLd, SIL2)</t>
+          <t>What functional safety level is required? (e.g. PLd, SIL2)</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -4071,7 +4071,7 @@
       </c>
       <c r="Q35" s="64" t="inlineStr">
         <is>
-          <t>Welche Bereiche rund um das Fahrzeug müssen durch Sicherheitssensorik abgedeckt werden?</t>
+          <t>Which areas must be covered by safety sensors?</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="Q37" s="64" t="inlineStr">
         <is>
-          <t>Gibt es ein bestehendes Flottenleitsystem, das kompatibel sein muss?</t>
+          <t>Is there an existing fleet management system that must be compatible?</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="Q38" s="64" t="inlineStr">
         <is>
-          <t>Welche Steuerungsarchitektur ist für die Flotte vorgesehen? (z. B. zentralisiert, dezentralisiert)</t>
+          <t>What control architecture is intended for the fleet? (centralised, decentralised)</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="Q39" s="64" t="inlineStr">
         <is>
-          <t>Muss das AGV den VDA-5050-Standard für Schnittstellen unterstützen?</t>
+          <t>Must the AGV support the VDA 5050 interface standard?</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="Q40" s="64" t="inlineStr">
         <is>
-          <t>Wie viele AGVs sollen gleichzeitig im Einsatz sein?</t>
+          <t>How many AGVs should be in simultaneous operation?</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="Q41" s="64" t="inlineStr">
         <is>
-          <t>Müssen AGVs verschiedener Hersteller im selben Bereich kooperieren können?</t>
+          <t>Must AGVs from different manufacturers be able to coexist in the same area?</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="Q42" s="64" t="inlineStr">
         <is>
-          <t>Mit welchen bestehenden Systemen muss das AGV integriert werden? (WMS, ERP, MES)</t>
+          <t>Which existing systems must the AGV integrate with? (WMS, ERP, MES)</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4389,7 +4389,7 @@
       </c>
       <c r="Q43" s="64" t="inlineStr">
         <is>
-          <t>Gibt es besondere Anforderungen an den Installationsprozess des AGV-Systems?</t>
+          <t>Are there requirements for the installation process of the AGV system?</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="Q44" s="64" t="inlineStr">
         <is>
-          <t>Wie einfach müssen spätere Anpassungen oder Erweiterungen möglich sein?</t>
+          <t>How easy must later modifications or expansions be?</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="Q46" s="64" t="inlineStr">
         <is>
-          <t>Welche speziellen Stationsanwendungen werden benötigt? (z. B. Ladestation, Übergabestation)</t>
+          <t>What special station applications are required? (e.g. charging station, transfer station)</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4555,7 +4555,7 @@
       </c>
       <c r="Q48" s="64" t="inlineStr">
         <is>
-          <t>Anzahl der Referenzprojekte des Anbieters (wird automatisch befüllt)</t>
+          <t>Number of reference projects from the supplier. (filled automatically)</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4615,7 +4615,7 @@
       </c>
       <c r="Q49" s="64" t="inlineStr">
         <is>
-          <t>Wie viele Wochen Vorlaufzeit bis zur Inbetriebnahme sind akzeptabel?</t>
+          <t>How many weeks lead time until commissioning is acceptable?</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4665,7 +4665,7 @@
       </c>
       <c r="Q50" s="64" t="inlineStr">
         <is>
-          <t>In welchen Ländern oder Regionen ist Service und Support erforderlich?</t>
+          <t>In which countries or regions is service and support required?</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="Q51" s="64" t="inlineStr">
         <is>
-          <t>Wie viele AGVs werden mindestens benötigt?</t>
+          <t>How many AGVs are needed as a minimum?</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="Q52" s="64" t="inlineStr">
         <is>
-          <t>Welches Budget steht für das AGV-Projekt zur Verfügung? (EUR)</t>
+          <t>What budget is available for the AGV project? (EUR)</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="Q54" s="64" t="inlineStr">
         <is>
-          <t>Soll das Fahrzeug auch manuell bedienbar sein?</t>
+          <t>Should the vehicle also be manually operable?</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -4840,7 +4840,7 @@
       </c>
       <c r="Q55" s="64" t="inlineStr">
         <is>
-          <t>In welcher Branche wird das AGV eingesetzt?</t>
+          <t>In which industry will the AGV be used?</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="Q56" s="64" t="inlineStr">
         <is>
-          <t>Wie wird das AGV vertrieben bzw. geliefert?</t>
+          <t>How is the AGV sold or delivered?</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="Q58" s="64" t="inlineStr">
         <is>
-          <t>Welcher AGV-Typ ist erforderlich? (wird automatisch aus der Ausschreibung erkannt)</t>
+          <t>What AGV type is required? (automatically detected from the document)</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="Q59" s="64" t="inlineStr">
         <is>
-          <t>In welchem Land befindet sich der Betriebsort?</t>
+          <t>In which country is the operating site located?</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="Q60" s="64" t="inlineStr">
         <is>
-          <t>Mitarbeiteranzahl des Herstellers (wird automatisch befüllt)</t>
+          <t>Number of employees at the manufacturer. (filled automatically)</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5075,7 +5075,7 @@
       </c>
       <c r="Q61" s="64" t="inlineStr">
         <is>
-          <t>Welche Zertifizierungen muss der Hersteller nachweisen? (z. B. ISO 9001)</t>
+          <t>Which certifications must the manufacturer hold? (e.g. ISO 9001)</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="Q62" s="64" t="inlineStr">
         <is>
-          <t>Welche Sprache(n) muss der Hersteller für Support und Dokumentation beherrschen?</t>
+          <t>Which language(s) must the manufacturer support for service and documentation?</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="Q63" s="64" t="inlineStr">
         <is>
-          <t>Hauptsitz des Herstellers (wird automatisch befüllt)</t>
+          <t>Manufacturer headquarters. (filled automatically)</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="Q64" s="64" t="inlineStr">
         <is>
-          <t>Gründungsjahr des Herstellers (wird automatisch befüllt)</t>
+          <t>Manufacturer founding year. (filled automatically)</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="Q4" s="64" t="inlineStr">
         <is>
-          <t>Bis zu welcher Höhe muss das Gerät Lasten anheben? Maximale Entnahmehöhe im Regal angeben (mm; z. B. 10.000 mm = 10 m für Hochregal).</t>
+          <t>How high must the device lift loads? Enter the maximum pick height in the rack. (mm; e.g. 10,000 mm = 10 m for high-bay storage)</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -5469,7 +5469,7 @@
       </c>
       <c r="Q5" s="64" t="inlineStr">
         <is>
-          <t>Wie hoch sind die niedrigsten Durchfahrten oder Türen im Betriebsbereich? (mm)</t>
+          <t>What is the height of the lowest doorways or passages in the operating area? (mm)</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="Q6" s="64" t="inlineStr">
         <is>
-          <t>Wird eine spezielle Gabelausführung benötigt? (z. B. Seitenschieber, Klammergreifer)</t>
+          <t>Is a special fork attachment required? (e.g. side-shift, clamp)</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -5563,7 +5563,7 @@
       </c>
       <c r="Q7" s="64" t="inlineStr">
         <is>
-          <t>Welcher Gabelabstand ist für die Ladungsträger erforderlich? (mm)</t>
+          <t>What fork spacing is required for the load carriers? (mm)</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="Q8" s="64" t="inlineStr">
         <is>
-          <t>Welcher Masttyp ist vorgesehen? (z. B. Duplex, Triplex, Vierstufig)</t>
+          <t>What mast type is intended? (e.g. duplex, triplex, quad)</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -5662,7 +5662,7 @@
       </c>
       <c r="Q9" s="64" t="inlineStr">
         <is>
-          <t>Wie breit sind die schmalsten Fahrwege in Ihrer Anlage? Das AGV muss in dieser Gangbreite fahren können (mm).</t>
+          <t>How wide are the narrowest aisles in your facility? The AGV must manoeuvre within this width. (mm; e.g. 1,800 mm for narrow-aisle operation)</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="Q10" s="64" t="inlineStr">
         <is>
-          <t>Ist VNA-Fähigkeit (Schmalgangbetrieb) erforderlich — oder explizit nicht gewünscht?</t>
+          <t>Is VNA (Very Narrow Aisle) capability required — or explicitly not desired?</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -5769,7 +5769,7 @@
       <c r="H12" s="52" t="n"/>
       <c r="Q12" s="64" t="inlineStr">
         <is>
-          <t>Welcher Antriebstyp ist vorgesehen? (z. B. Gegengewichtstapler, Schubmast, VNA)</t>
+          <t>What drive type is intended? (e.g. counterbalanced, reach truck, VNA)</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -5833,7 +5833,7 @@
       </c>
       <c r="Q14" s="64" t="inlineStr">
         <is>
-          <t>Wie präzise muss das AMR Lasten seitlich absetzen? (mm laterale Abweichung)</t>
+          <t>How precisely must the AMR deposit loads laterally? (mm)</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="Q15" s="64" t="inlineStr">
         <is>
-          <t>Wie präzise muss das AMR Lasten in der Tiefe absetzen? (mm)</t>
+          <t>How precisely must the AMR deposit loads in depth? (mm)</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="Q16" s="64" t="inlineStr">
         <is>
-          <t>Wie präzise muss das AMR Lasten winkelgenau absetzen? (Grad)</t>
+          <t>How precisely must the AMR deposit loads angularly? (degrees)</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="Q17" s="64" t="inlineStr">
         <is>
-          <t>Welche seitliche Präzision ist bei der Lastaufnahme erforderlich? (mm)</t>
+          <t>What lateral precision is required when picking up loads? (mm)</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -6016,7 +6016,7 @@
       </c>
       <c r="Q18" s="64" t="inlineStr">
         <is>
-          <t>Welche Tiefenpräzision ist bei der Kommissionierung erforderlich? (mm)</t>
+          <t>What depth precision is required during order picking? (mm)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="Q19" s="64" t="inlineStr">
         <is>
-          <t>Welche Winkelpräzision ist bei der Kommissionierung erforderlich? (Grad)</t>
+          <t>What angular precision is required during order picking? (degrees)</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -6112,7 +6112,7 @@
       </c>
       <c r="Q21" s="64" t="inlineStr">
         <is>
-          <t>Müssen die Gabeln seitenverschiebbar oder schwimmend gelagert sein?</t>
+          <t>Must the forks be laterally shiftable or free-floating?</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -6156,7 +6156,7 @@
       <c r="I22" s="50" t="n"/>
       <c r="Q22" s="64" t="inlineStr">
         <is>
-          <t>Muss das Gerät Lasten übereinander stapeln können?</t>
+          <t>Must the device be able to stack loads on top of each other?</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -6198,7 +6198,7 @@
       </c>
       <c r="Q23" s="64" t="inlineStr">
         <is>
-          <t>Wie soll die Lastaufnahme erkannt werden?</t>
+          <t>How should load pickup be detected?</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="Q24" s="64" t="inlineStr">
         <is>
-          <t>Sind integrierte Barcode-Scanner für die Lastidentifikation erforderlich?</t>
+          <t>Are integrated barcode scanners for load identification required?</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="Q25" s="64" t="inlineStr">
         <is>
-          <t>Muss das AGV Bestände im Regal automatisch scannen können?</t>
+          <t>Must the AGV be able to automatically scan inventory in the racks?</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="Q27" s="64" t="inlineStr">
         <is>
-          <t>Muss das AGV Lasten in Lkw-Trailer einfahren und beladen können?</t>
+          <t>Must the AGV be able to enter and load truck trailers?</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -6375,7 +6375,7 @@
       </c>
       <c r="Q28" s="64" t="inlineStr">
         <is>
-          <t>Muss das AGV Lasten aus Lkw-Trailern entnehmen können?</t>
+          <t>Must the AGV be able to unload from truck trailers?</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -6432,7 +6432,7 @@
       </c>
       <c r="Q30" s="64" t="inlineStr">
         <is>
-          <t>Welches Führungskonzept soll das Regalfahrzeug im VNA-Bereich nutzen?</t>
+          <t>What guidance concept should the racking vehicle use in the VNA aisle?</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="Q31" s="64" t="inlineStr">
         <is>
-          <t>Ist ein Stromversorgungssystem über Schienenschleifer (Busbar) vorgesehen?</t>
+          <t>Is a rail-based power supply system (busbar) planned?</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -6680,7 +6680,7 @@
       </c>
       <c r="Q4" s="64" t="inlineStr">
         <is>
-          <t>Wie hoch ist das maximale Gesamtgewicht des Anhängerzuges? (kg; Summe aller Anhänger inkl. Ladung)</t>
+          <t>What is the maximum total weight of the train? (kg; sum of all trailers including load; e.g. 5,000 kg)</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -6734,7 +6734,7 @@
       </c>
       <c r="Q5" s="64" t="inlineStr">
         <is>
-          <t>Wie viele Anhänger müssen gleichzeitig gezogen werden können?</t>
+          <t>How many trailers must be able to be towed simultaneously?</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -6781,7 +6781,7 @@
       </c>
       <c r="Q6" s="64" t="inlineStr">
         <is>
-          <t>Welche Kupplungsart verwenden die vorhandenen oder geplanten Anhänger?</t>
+          <t>What coupling type do the existing or planned trailers use?</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -6832,7 +6832,7 @@
       </c>
       <c r="Q7" s="64" t="inlineStr">
         <is>
-          <t>Muss der Tugger Anhänger automatisch ankuppeln können?</t>
+          <t>Must the tugger be able to automatically couple trailers?</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="Q8" s="64" t="inlineStr">
         <is>
-          <t>Welche Positioniertoleranz ist beim automatischen Ankuppeln akzeptabel? (mm)</t>
+          <t>What positioning tolerance is acceptable for automatic coupling? (mm)</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -6917,7 +6917,7 @@
       </c>
       <c r="Q9" s="64" t="inlineStr">
         <is>
-          <t>Welche Zuganordnung ist vorgesehen? (z. B. Anhänger in Reihe, Karussellanordnung)</t>
+          <t>What train configuration is intended? (e.g. trailers in line, carousel)</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="Q10" s="64" t="inlineStr">
         <is>
-          <t>Wie soll die Lastübergabe am Anhänger erfolgen?</t>
+          <t>How should the load handover at the trailer be performed?</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="Q12" s="64" t="inlineStr">
         <is>
-          <t>Welche Anhängertypen sollen verwendet werden?</t>
+          <t>Which trailer types will be used?</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -7057,7 +7057,7 @@
       </c>
       <c r="Q13" s="64" t="inlineStr">
         <is>
-          <t>Welche Lenktechnologie verwenden die Anhänger? (z. B. passive Lenkung, aktive Lenkung)</t>
+          <t>What steering technology do the trailers use? (e.g. passive steering, active steering)</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="Q15" s="64" t="inlineStr">
         <is>
-          <t>Welche Art von Fahrstrecke ist geplant? (feste Route oder flexible Route)</t>
+          <t>What type of route is planned? (fixed route, flexible route)</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -7156,7 +7156,7 @@
       </c>
       <c r="Q16" s="64" t="inlineStr">
         <is>
-          <t>Wie sollen Fahrrouten programmiert oder angepasst werden?</t>
+          <t>How should routes be programmed or adjusted?</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="Q17" s="64" t="inlineStr">
         <is>
-          <t>Wie sollen Kreuzungssituationen zwischen mehreren AGVs gehandhabt werden?</t>
+          <t>How should intersection situations between multiple AGVs be handled?</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="Q18" s="64" t="inlineStr">
         <is>
-          <t>Wie breit sind die schmalsten Fahrwege in Ihrer Anlage? Das AGV muss in dieser Gangbreite fahren können (mm).</t>
+          <t>How wide are the narrowest aisles in your facility? The AGV must manoeuvre within this width. (mm; e.g. 1,800 mm for narrow-aisle operation)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="Q19" s="64" t="inlineStr">
         <is>
-          <t>Wie viel Platz steht in Kurven zur Verfügung? (mm; der Wenderadius des Fahrzeugs muss kleiner sein)</t>
+          <t>How much space is available for cornering? (mm; vehicle turning radius must be smaller)</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -7356,7 +7356,7 @@
       </c>
       <c r="Q20" s="64" t="inlineStr">
         <is>
-          <t>Wie breit sind die schmalsten Durchfahrten im gesamten Fahrtbereich des Tuggers inkl. Anhänger? (mm)</t>
+          <t>How wide are the narrowest passages in the entire travel area including trailers? (mm)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="Q4" s="64" t="inlineStr">
         <is>
-          <t>Welche Arbeitsabläufe soll das AMR unterstützen?</t>
+          <t>What workflows should the AMR support?</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -7599,7 +7599,7 @@
       </c>
       <c r="Q5" s="64" t="inlineStr">
         <is>
-          <t>Ist ein physisches Gittersystem (z. B. Lagerroboter-Raster) Teil der Lösung?</t>
+          <t>Is a physical grid system (e.g. storage robot grid) part of the solution?</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -7645,7 +7645,7 @@
       </c>
       <c r="Q6" s="64" t="inlineStr">
         <is>
-          <t>Muss das AMR Lasten während der Fahrt drehen können?</t>
+          <t>Must the AMR be able to rotate loads during travel?</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="Q7" s="64" t="inlineStr">
         <is>
-          <t>Welcher Mechanismus soll das AMR zum Greifen oder Kommissionieren verwenden?</t>
+          <t>What mechanism should the AMR use for picking or gripping?</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -7756,7 +7756,7 @@
       </c>
       <c r="Q9" s="64" t="inlineStr">
         <is>
-          <t>Bis zu welcher Höhe muss das AMR Lasten oder Regale anheben? (mm)</t>
+          <t>How high must the AMR lift loads or shelving units? (mm)</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -7810,7 +7810,7 @@
       </c>
       <c r="Q10" s="64" t="inlineStr">
         <is>
-          <t>Wie viel Bodenfreiheit wird mindestens benötigt? (mm; z. B. für Bodenunebenheiten oder Schwellen)</t>
+          <t>What minimum ground clearance is required? (mm; e.g. for floor unevenness)</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -7853,7 +7853,7 @@
       </c>
       <c r="Q11" s="64" t="inlineStr">
         <is>
-          <t>Muss das AMR mit pin-kompatiblen Lagerregalen arbeiten können?</t>
+          <t>Must the AMR work with pin-compatible storage racks?</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="Q12" s="64" t="inlineStr">
         <is>
-          <t>Muss das AMR Paletten ohne Gabelöffnungen (Vollpaletten) aufnehmen können?</t>
+          <t>Must the AMR be able to pick up pallets without fork openings?</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -7938,7 +7938,7 @@
       </c>
       <c r="Q13" s="64" t="inlineStr">
         <is>
-          <t>Welches Aufbaumodul ist erforderlich? (z. B. Förderband, Hubtisch, Greifarme)</t>
+          <t>What top module is required? (e.g. conveyor belt, lifting table, robotic arms)</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="Q14" s="64" t="inlineStr">
         <is>
-          <t>In welchem Höhenbereich muss das AMR Wagen oder Ladungsträger aufnehmen? (mm)</t>
+          <t>At what height range must the AMR pick up carts or carriers? (mm)</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="Q16" s="64" t="inlineStr">
         <is>
-          <t>Wie viel Platz steht für Drehbewegungen zur Verfügung? (mm; der Wendekreis des AMR muss kleiner sein)</t>
+          <t>How much space is available for turning movements? (mm; turning radius must be smaller)</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -8099,7 +8099,7 @@
       </c>
       <c r="Q19" s="64" t="inlineStr">
         <is>
-          <t>Welche Tiefenpräzision ist bei der Kommissionierung erforderlich? (mm)</t>
+          <t>What depth precision is required during order picking? (mm)</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -8142,7 +8142,7 @@
       </c>
       <c r="Q20" s="64" t="inlineStr">
         <is>
-          <t>Welche Winkelpräzision ist bei der Kommissionierung erforderlich? (Grad)</t>
+          <t>What angular precision is required during order picking? (degrees)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -8185,7 +8185,7 @@
       </c>
       <c r="Q21" s="64" t="inlineStr">
         <is>
-          <t>Wie präzise muss das AMR Lasten seitlich absetzen? (mm laterale Abweichung)</t>
+          <t>How precisely must the AMR deposit loads laterally? (mm)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -8228,7 +8228,7 @@
       </c>
       <c r="Q22" s="64" t="inlineStr">
         <is>
-          <t>Wie präzise muss das AMR Lasten in der Tiefe absetzen? (mm)</t>
+          <t>How precisely must the AMR deposit loads in depth? (mm)</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -8271,7 +8271,7 @@
       </c>
       <c r="Q23" s="64" t="inlineStr">
         <is>
-          <t>Wie präzise muss das AMR Lasten winkelgenau absetzen? (Grad)</t>
+          <t>How precisely must the AMR deposit loads angularly? (degrees)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="Q25" s="64" t="inlineStr">
         <is>
-          <t>Welches Lagersystem soll das AMR bedienen?</t>
+          <t>What storage system should the AMR serve?</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="Q26" s="64" t="inlineStr">
         <is>
-          <t>Wie hoch sind die Lagerregale, die das AMR bedienen soll? (mm)</t>
+          <t>How high are the storage racks the AMR should serve? (mm)</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -8425,7 +8425,7 @@
       </c>
       <c r="Q27" s="64" t="inlineStr">
         <is>
-          <t>Wie groß ist der Grundriss der Lagereinheiten? (mm)</t>
+          <t>What is the footprint of the storage units? (mm)</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -8468,7 +8468,7 @@
       </c>
       <c r="Q28" s="64" t="inlineStr">
         <is>
-          <t>Wie groß ist die minimale Lagerfläche für das AMR-System? (m²)</t>
+          <t>What is the minimum storage area for the AMR system? (m²)</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -8541,7 +8541,7 @@
       </c>
       <c r="Q30" s="64" t="inlineStr">
         <is>
-          <t>Wie viele Kommissionierungen pro Stunde sind mindestens erforderlich?</t>
+          <t>How many picks per hour are required as a minimum?</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="Q31" s="64" t="inlineStr">
         <is>
-          <t>Auf welcher Basis wird der Durchsatz gemessen?</t>
+          <t>On what basis is throughput measured?</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -8626,7 +8626,7 @@
       </c>
       <c r="Q32" s="64" t="inlineStr">
         <is>
-          <t>Wie viele AMRs müssen gleichzeitig an einer Station arbeiten können?</t>
+          <t>How many AMRs must be able to work at one station simultaneously?</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="Q33" s="64" t="inlineStr">
         <is>
-          <t>Wie viele Auftragspositionen sollen pro Fahrt abgearbeitet werden?</t>
+          <t>How many order lines should be processed per trip?</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -8707,7 +8707,7 @@
       </c>
       <c r="Q34" s="64" t="inlineStr">
         <is>
-          <t>Sollen AMRs verschiedene Aufgabentypen im Wechsel abarbeiten können?</t>
+          <t>Should AMRs be able to alternate between different task types?</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -8750,7 +8750,7 @@
       </c>
       <c r="Q35" s="64" t="inlineStr">
         <is>
-          <t>Wie wichtig ist eine hohe Lagerplatzdichte für Ihr System?</t>
+          <t>How important is high storage density for your system?</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -8788,7 +8788,7 @@
       </c>
       <c r="Q36" s="64" t="inlineStr">
         <is>
-          <t>Muss die Arbeitshöhe für Mitarbeiter ergonomisch anpassbar sein?</t>
+          <t>Must the working height be ergonomically adjustable for operators?</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -8826,7 +8826,7 @@
       </c>
       <c r="Q37" s="64" t="inlineStr">
         <is>
-          <t>Ist ein Display oder Bedienpanel am Fahrzeug erforderlich?</t>
+          <t>Is a display or control panel on the vehicle required?</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="Q38" s="64" t="inlineStr">
         <is>
-          <t>Muss die Anzeige am Fahrzeug mehrsprachig sein?</t>
+          <t>Must the display support multiple languages?</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="Q39" s="64" t="inlineStr">
         <is>
-          <t>Sind spielerische Motivationselemente für Mitarbeiter gewünscht?</t>
+          <t>Are gamification elements for operator motivation desired?</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -8959,7 +8959,7 @@
       </c>
       <c r="Q41" s="64" t="inlineStr">
         <is>
-          <t>Welcher Behältertyp soll auf dem AMR transportiert werden?</t>
+          <t>What container type should be transported on the AMR?</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -9002,7 +9002,7 @@
       </c>
       <c r="Q42" s="64" t="inlineStr">
         <is>
-          <t>Wie viele Behälter soll das AMR gleichzeitig transportieren?</t>
+          <t>How many containers should the AMR transport simultaneously?</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -9058,7 +9058,7 @@
       </c>
       <c r="Q44" s="64" t="inlineStr">
         <is>
-          <t>Ist eine direkte native Integration mit dem Warehouse-Management-System erforderlich?</t>
+          <t>Is a direct native integration with the Warehouse Management System required?</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">

</xml_diff>

<commit_message>
Refactor: remove result_card from AP0 boundary (OI-44 + M2)
AP0 xlsx:
- result_card column cleared (concept retired per OI-52 decision)

generate_all.py / field_spec.py / fields.json:
- result_card no longer read, emitted, or stored

matching.py:
- _RESULT_CARD_FIELDS constant removed
- to_dict() now includes all level != CONTEXT fields (AP0-driven)
  instead of an explicit result_card list

app.py:
- result_card removed from /api/field-meta response

tests:
- test_T_DM_04: asserts result_card absent from field-meta (regression guard)
- test_T_DM_05: asserts debug.html's three field names always in to_dict()

187 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -2596,9 +2596,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -2640,8 +2640,6 @@
           <t>Fields applying to ALL AGV/AMR subtypes — written into base_model_extensions for every base model. Universal fields are consolidated here: power, gradient, floor flatness, stop accuracy, station applications, fleet size. ● = added/changed by Claude. v0.7: navigation_type + infrastructure_required → Cond. K.O.; Company/Product fields added.. Colour = level (red K.O. · orange Cond. K.O. · yellow Scoring · green Context).</t>
         </is>
       </c>
-      <c r="C1" s="64" t="n"/>
-      <c r="G1" s="64" t="n"/>
       <c r="Q1" s="64" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1" s="57">
@@ -2742,8 +2740,6 @@
           <t>── NAVIGATION &amp; INFRASTRUCTURE</t>
         </is>
       </c>
-      <c r="C3" s="64" t="n"/>
-      <c r="G3" s="64" t="n"/>
       <c r="Q3" s="64" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="57">
@@ -2782,9 +2778,6 @@
           <t>KO_SUBSET</t>
         </is>
       </c>
-      <c r="O4" t="b">
-        <v>1</v>
-      </c>
       <c r="Q4" s="64" t="inlineStr">
         <is>
           <t>What navigation type is intended or allowed? (e.g. Natural Feature/SLAM, magnetic tape, QR code)</t>
@@ -2972,8 +2965,6 @@
           <t>── LOAD HANDLING</t>
         </is>
       </c>
-      <c r="C9" s="64" t="n"/>
-      <c r="G9" s="64" t="n"/>
       <c r="Q9" s="64" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="57">
@@ -3019,9 +3010,6 @@
       <c r="N10" t="n">
         <v>50000</v>
       </c>
-      <c r="O10" t="b">
-        <v>1</v>
-      </c>
       <c r="Q10" s="64" t="inlineStr">
         <is>
           <t>What is the maximum load weight per carrier? The AGV must be able to carry at least this weight.</t>
@@ -3129,8 +3117,6 @@
           <t>── DIMENSIONS &amp; ENVIRONMENT</t>
         </is>
       </c>
-      <c r="C13" s="64" t="n"/>
-      <c r="G13" s="64" t="n"/>
       <c r="Q13" s="64" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="57">
@@ -3165,9 +3151,6 @@
           <t>Top travel speed (capture rated/unloaded if only one given). Source: spec table. Implies cycle time; check safety-derated speed too.</t>
         </is>
       </c>
-      <c r="O14" t="b">
-        <v>1</v>
-      </c>
       <c r="Q14" s="64" t="inlineStr">
         <is>
           <t>What maximum speed should the AGV achieve? (m/s)</t>
@@ -3628,8 +3611,6 @@
           <t>── ACCURACY</t>
         </is>
       </c>
-      <c r="C24" s="64" t="n"/>
-      <c r="G24" s="64" t="n"/>
       <c r="Q24" s="64" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="57">
@@ -3695,8 +3676,6 @@
           <t>── POWER</t>
         </is>
       </c>
-      <c r="C26" s="64" t="n"/>
-      <c r="G26" s="64" t="n"/>
       <c r="Q26" s="64" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="57">
@@ -3784,9 +3763,6 @@
       <c r="K28" t="n">
         <v>8</v>
       </c>
-      <c r="O28" t="b">
-        <v>1</v>
-      </c>
       <c r="Q28" s="64" t="inlineStr">
         <is>
           <t>How many hours of operating time per charge are required as a minimum? (h)</t>
@@ -3876,9 +3852,6 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="O30" t="b">
-        <v>1</v>
-      </c>
       <c r="Q30" s="64" t="inlineStr">
         <is>
           <t>Must the AGV autonomously navigate to the charging station and charge itself?</t>
@@ -3934,8 +3907,6 @@
           <t>── SAFETY &amp; CERTIFICATION</t>
         </is>
       </c>
-      <c r="C32" s="64" t="n"/>
-      <c r="G32" s="64" t="n"/>
       <c r="Q32" s="64" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="57">
@@ -4086,8 +4057,6 @@
           <t>── FLEET &amp; INTEGRATION</t>
         </is>
       </c>
-      <c r="C36" s="64" t="n"/>
-      <c r="G36" s="64" t="n"/>
       <c r="Q36" s="64" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="57">
@@ -4219,9 +4188,6 @@
           <t>bool_cond</t>
         </is>
       </c>
-      <c r="O39" t="b">
-        <v>1</v>
-      </c>
       <c r="Q39" s="64" t="inlineStr">
         <is>
           <t>Must the AGV support the VDA 5050 interface standard?</t>
@@ -4446,8 +4412,6 @@
           <t>── STATIONS</t>
         </is>
       </c>
-      <c r="C45" s="64" t="n"/>
-      <c r="G45" s="64" t="n"/>
       <c r="Q45" s="64" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="57">
@@ -4503,8 +4467,6 @@
           <t>── COMMERCIAL</t>
         </is>
       </c>
-      <c r="C47" s="64" t="n"/>
-      <c r="G47" s="64" t="n"/>
       <c r="Q47" s="64" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="57">
@@ -4550,9 +4512,6 @@
       <c r="K48" t="n">
         <v>20</v>
       </c>
-      <c r="O48" t="b">
-        <v>1</v>
-      </c>
       <c r="Q48" s="64" t="inlineStr">
         <is>
           <t>Number of reference projects from the supplier. (filled automatically)</t>
@@ -4610,9 +4569,6 @@
       <c r="L49" t="n">
         <v>52</v>
       </c>
-      <c r="O49" t="b">
-        <v>1</v>
-      </c>
       <c r="Q49" s="64" t="inlineStr">
         <is>
           <t>How many weeks lead time until commissioning is acceptable?</t>
@@ -4660,9 +4616,6 @@
           <t>KO_SUBSET</t>
         </is>
       </c>
-      <c r="O50" t="b">
-        <v>1</v>
-      </c>
       <c r="Q50" s="64" t="inlineStr">
         <is>
           <t>In which countries or regions is service and support required?</t>
@@ -4765,8 +4718,6 @@
           <t>── CONTEXT</t>
         </is>
       </c>
-      <c r="C53" s="64" t="n"/>
-      <c r="G53" s="64" t="n"/>
       <c r="Q53" s="64" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="57">
@@ -5261,8 +5212,6 @@
           <t>Forklift-specific fields only (universal fields live in SHARED). Pick/drop accuracy ordered lateral·depth·angle. ● = changed/added by Claude. Combine with SHARED.</t>
         </is>
       </c>
-      <c r="C1" s="64" t="n"/>
-      <c r="G1" s="64" t="n"/>
       <c r="Q1" s="64" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1" s="57">
@@ -5363,8 +5312,6 @@
           <t>── MAST &amp; LIFTING</t>
         </is>
       </c>
-      <c r="C3" s="64" t="n"/>
-      <c r="G3" s="64" t="n"/>
       <c r="Q3" s="64" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="57">
@@ -5410,9 +5357,6 @@
       <c r="N4" t="n">
         <v>30</v>
       </c>
-      <c r="O4" t="b">
-        <v>1</v>
-      </c>
       <c r="Q4" s="64" t="inlineStr">
         <is>
           <t>How high must the device lift loads? Enter the maximum pick height in the rack. (mm; e.g. 10,000 mm = 10 m for high-bay storage)</t>
@@ -5657,9 +5601,6 @@
       <c r="N9" t="n">
         <v>5</v>
       </c>
-      <c r="O9" t="b">
-        <v>1</v>
-      </c>
       <c r="Q9" s="64" t="inlineStr">
         <is>
           <t>How wide are the narrowest aisles in your facility? The AGV must manoeuvre within this width. (mm; e.g. 1,800 mm for narrow-aisle operation)</t>
@@ -5725,8 +5666,6 @@
           <t>── DRIVE</t>
         </is>
       </c>
-      <c r="C11" s="64" t="n"/>
-      <c r="G11" s="64" t="n"/>
       <c r="Q11" s="64" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="57">
@@ -5784,8 +5723,6 @@
           <t>── PICK &amp; DROP (order: lateral · depth · angle)</t>
         </is>
       </c>
-      <c r="C13" s="64" t="n"/>
-      <c r="G13" s="64" t="n"/>
       <c r="Q13" s="64" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="57">
@@ -6074,8 +6011,6 @@
           <t>── HANDLING CAPABILITY</t>
         </is>
       </c>
-      <c r="C20" s="64" t="n"/>
-      <c r="G20" s="64" t="n"/>
       <c r="Q20" s="64" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="57">
@@ -6294,8 +6229,6 @@
           <t>── TRAILER / DOCK</t>
         </is>
       </c>
-      <c r="C26" s="64" t="n"/>
-      <c r="G26" s="64" t="n"/>
       <c r="Q26" s="64" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="57">
@@ -6390,8 +6323,6 @@
           <t>── AGV (RAIL/WIRE) ONLY</t>
         </is>
       </c>
-      <c r="C29" s="64" t="n"/>
-      <c r="G29" s="64" t="n"/>
       <c r="Q29" s="64" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="57">
@@ -6529,8 +6460,6 @@
           <t>Tugger-specific fields, deepened from Vecna / DS Automotion / LKE research — trailer compatibility &amp; steering tech, aisle width, turning radius, auto-hitch + tolerance. ● = added by Claude. Combine with SHARED. v0.7: auto_hitch → Cond. K.O.; tugger_min_aisle_width_mm added.</t>
         </is>
       </c>
-      <c r="C1" s="64" t="n"/>
-      <c r="G1" s="64" t="n"/>
       <c r="Q1" s="64" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1" s="57">
@@ -6631,8 +6560,6 @@
           <t>── TOWING</t>
         </is>
       </c>
-      <c r="C3" s="64" t="n"/>
-      <c r="G3" s="64" t="n"/>
       <c r="Q3" s="64" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="57">
@@ -6974,8 +6901,6 @@
           <t>── TRAILER / CART</t>
         </is>
       </c>
-      <c r="C11" s="64" t="n"/>
-      <c r="G11" s="64" t="n"/>
       <c r="Q11" s="64" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="57">
@@ -7072,8 +6997,6 @@
           <t>── ROUTING &amp; MANEUVERING</t>
         </is>
       </c>
-      <c r="C14" s="64" t="n"/>
-      <c r="G14" s="64" t="n"/>
       <c r="Q14" s="64" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="57">
@@ -7412,8 +7335,6 @@
           <t>Unified free-navigating AMR sheet — merges the former Undercarriage + Goods-to-Person + Picking subtypes into ONE category (same hardware, different workflow). The workflow is now a PROPERTY (workflow_capability, grid_required, rotation_capable, picking_mechanism), not a hard category. Overlapping throughput fields consolidated into throughput_picks_per_hour + throughput_basis. ● = added/changed by Claude. Combine with SHARED.</t>
         </is>
       </c>
-      <c r="C1" s="64" t="n"/>
-      <c r="G1" s="64" t="n"/>
       <c r="Q1" s="64" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1" s="57">
@@ -7514,8 +7435,6 @@
           <t>── WORKFLOW MODE (property-based — replaces the old Undercarriage / G2P / Picking split)</t>
         </is>
       </c>
-      <c r="C3" s="64" t="n"/>
-      <c r="G3" s="64" t="n"/>
       <c r="Q3" s="64" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="57">
@@ -7707,8 +7626,6 @@
           <t>── LOAD HANDLING &amp; LIFT</t>
         </is>
       </c>
-      <c r="C8" s="64" t="n"/>
-      <c r="G8" s="64" t="n"/>
       <c r="Q8" s="64" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="57">
@@ -7991,8 +7908,6 @@
           <t>── MOVEMENT</t>
         </is>
       </c>
-      <c r="C15" s="64" t="n"/>
-      <c r="G15" s="64" t="n"/>
       <c r="Q15" s="64" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="57">

</xml_diff>

<commit_message>
IK Sprint Phase 3: IK-Felder in AP0 + generate_all.py B1-Fix + app.py Change B (SA-approved)
- AP0 xlsx: neuer Tab FoodBev_Refrigeration mit 12 IK-Feldern (entity=Base Model, scope=FoodBev:Refrigeration)
- AP0 ③ Scope Registry: tab_name + variant_guide_json für FoodBev:Refrigeration
- generate_all.py: build_scope_classification_template B1-Fix (single-leaf domains via variant_guides), @SCOPE_VARIANTS sentinel, required_served_categories in _4A_FIELDS
- IK-README: vollständiges Domänenwissen (Kältemittel, COP, EN 378, Terminologie DE/EN)
- app.py: required_served_categories aus Pass 4a für Single-Leaf-Domains (AP0-driven, kein Hardcode)
- CSV-Migration: agv_type=Industrial Refrigeration + served_categories für GEA/Güntner/BITZER
- 241 Tests grün

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Representatives" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Vehicle Types" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Field Fallbacks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="FoodBev_Refrigeration" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -904,7 +905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2649,6 +2650,660 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fields applying to Industrial Refrigeration (FoodBev domain) — written into base_model_extensions. 12 IK fields: 6 KO + 6 Cond. K.O. Colour = level (red K.O. · orange Cond. K.O.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Allowed Values</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>LLM Hint</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Matching Operator</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Scoring Weight</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Score Function</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Score Threshold A</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Score Threshold B</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Plausibility Min</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Plausibility Max</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>result_card</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Display Mode</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>UI Hint</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>UUID</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Value if Null</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>served_categories</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Multi-Select</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>@SCOPE_VARIANTS:FoodBev:Refrigeration</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>K.O.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Extract ALL categories of refrigeration applications this supplier can serve. Do NOT assume from product name alone — extract only if stated explicitly. NULL RULE: if not explicitly stated, return null.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>KO_SUBSET</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>23992ff7-c679-4328-971a-e0ad5700af80</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cooling_capacity_kw</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>K.O.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Extract the MAXIMUM total cooling capacity in kW. Use the highest stated value. Do NOT convert from tons of refrigeration unless the document provides an explicit conversion. NULL RULE: return null if no explicit kW or TR figure is found.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>KO_IF_LT</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
+        <v>100000</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>b8e6446a-07dd-4414-91c5-55d2646651b8</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>temperature_min_celsius</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>K.O.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Extract the MINIMUM evaporation or supply temperature the system can achieve in °C. Use the lowest (most negative) stated temperature target. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>KO_IF_GT</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>-60</v>
+      </c>
+      <c r="N5" t="n">
+        <v>15</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>833fb224-f218-4b28-8719-591a0ba86483</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>refrigerant_types</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Multi-Select</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>R717|R744|R290|R134a|R32|R404A|R452A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>K.O.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Extract ALL refrigerant types supported by this system. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>KO_SUBSET</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>59b9c33b-833a-4026-8061-2fab3a68de0c</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>certifications_ik</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Multi-Select</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PED|ATEX|EN 378|F-Gas</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>K.O.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Extract ALL relevant certifications held by this system. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>KO_SUBSET</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>c7989fc1-f256-4159-9c4c-ae3f481836ff</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>cop_efficiency</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>K.O.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Extract the COP (Coefficient of Performance) at rated conditions. Use the highest stated COP. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>KO_IF_LT</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N8" t="n">
+        <v>15</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>b5204d0e-9069-4f9b-844a-b464bf2c2ef7</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cooling_medium</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Dropdown</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>glycol|water|direct</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Cond. K.O.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Extract the cooling medium used: glycol circuit, water, or direct expansion. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>KO_IF_NEQ</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>80fb3a63-341f-47b0-85ec-b41c8169f7af</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>temperature_stability_k</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Cond. K.O.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Extract the maximum temperature fluctuation tolerance in Kelvin. Lower is better. NULL RULE: return null if no explicit tolerance value is stated.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>KO_IF_GT</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N10" t="n">
+        <v>10</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>d4acded7-017e-4328-a2f4-115095a717b1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>room_volume_m3_max</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Cond. K.O.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Extract the MAXIMUM room volume in m³ this system can handle. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>KO_IF_LT</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>fde5ac60-1669-4543-89ec-03e02a2930b4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>humidity_control_capable</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Cond. K.O.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Does this system provide active humidity control? Only mark true if explicitly confirmed. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>KO_BOOL_REQUIRED</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>b6921aa9-6d37-4432-9e26-b0b321052a07</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>blast_freeze_capacity_kg_h</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>kg/h</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Cond. K.O.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Extract the blast freezing throughput capacity in kg/h. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>KO_IF_LT</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>100000</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>fb9c7834-e48d-40d0-a0ef-4d5e8d1d75d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>pulldown_time_h</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Cond. K.O.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Base Model</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Extract the required pulldown time in hours (time to reach target temperature). Lower is better for supplier. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>KO_IF_GT</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>48</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>265424b5-ee01-4bc4-9c3f-072d53ff64dd</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4201,7 +4856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4273,6 +4928,11 @@
       <c r="N1" t="inlineStr">
         <is>
           <t>vna_hint</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>variant_guide_json</t>
         </is>
       </c>
     </row>
@@ -4510,6 +5170,11 @@
           <t>Refrigeration Shared</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FoodBev_Refrigeration</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>✓</t>
@@ -4525,9 +5190,19 @@
           <t>Industrial Refrigeration</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>kälteanlage, kältetechnik, refrigeration, industrial cooling, cold store, deep freeze, blast freezer, prozesskühlung, tiefkühlung, kühlhaus</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Process Cooling, Cold Store, Deep Freeze</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>{"Process Cooling": "System actively cools process media (glycol circuits, milk, fermentation tanks, process water) in food or beverage production. Temperature range typically above freezing (+2°C to +15°C). Signals: Prozesskühlung, Brauerei, Milchkühlung, Gärung, process water, glycol chiller", "Cold Store": "System maintains a refrigerated room or warehouse for fresh product storage. Temperature range above freezing (+0°C to +8°C). Signals: Kühllager, Kühlhaus, cold store, cold room, fresh produce storage, Frischwarenlager", "Deep Freeze": "System freezes or maintains frozen products at temperatures well below freezing (-18°C to -40°C). Includes blast freezers and deep-freeze warehouses. Signals: Tiefkühlung, Tiefkühlanlage, Schockfrostung, blast freezer, deep freeze, frozen storage, Gefrieranlage"}</t>
         </is>
       </c>
     </row>
@@ -5460,9 +6135,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -5475,7 +6150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T53"/>
+  <dimension ref="A1:S53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="57" min="1" max="1"/>

</xml_diff>

<commit_message>
IK Sprint Phase 4: agv_type → product_type rename (SA-approved)
Purely mechanical rename across 58 files: AP0 xlsx, generate_all.py,
all src/*, app.py, sync_airtable.py, templates, airtable scripts,
historical scripts, 7 test files, 18 golden/fixture/run JSONs.
241 tests green. Airtable field rename pending (manual UI step).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -1458,7 +1458,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>agv_type</t>
+          <t>product_type</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4654,7 +4654,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>agv_type</t>
+          <t>product_type</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>agv_type</t>
+          <t>product_type</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -6135,8 +6135,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9641,7 +9641,7 @@
       </c>
       <c r="G4" s="68" t="inlineStr">
         <is>
-          <t>Total towed load in kg. [TUGGER ONLY] — output null unless required_agv_type is 'Tugger AGV'. Source: 'Schleppkraft / towing capacity'.</t>
+          <t>Total towed load in kg. [TUGGER ONLY] — output null unless required_product_type is 'Tugger AGV'. Source: 'Schleppkraft / towing capacity'.</t>
         </is>
       </c>
       <c r="H4" s="52" t="inlineStr">

</xml_diff>

<commit_message>
IK Sprint Phase 5: cleanup + IK golden tests + Güntner data fix (SA-approved)
SA findings F3–F6 resolved; 245 tests green.

Changes:
- app.py: write canonical product_type back to agv_criteria after line 1051 (F3)
- src/matching.py: fix _op_gt message to symmetric format (F5, cosmetic)
- scripts/generate_all.py: ValueError assertion for single-leaf domain missing variant_guides (F6)
- src/tender_store.py: remove is_agv_amr from _BASIC_INFO_KEYS (F4/OI-77 partial)
- templates/debug.html: remove is_agv_amr from skipKeys dead code (F4/OI-77 partial)
- templates/index.html + AP0 xlsx: Round-1 UI fixes (cop_efficiency unit=COP, certifications_ik UI hint)
- data/raw/base_model_extensions.csv: Güntner temperature_min_celsius 0.0 → -30.0 (spec: GASC datasheet doc 1846275M)
- tests: 3 IK golden fixtures (tender_006/007/008) + temperature KO direction test

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -2979,6 +2979,11 @@
           <t>KO_SUBSET</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Required safety certifications for the refrigeration system (e.g. EN 378, PED, ATEX for explosive atmospheres, F-Gas regulation)</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr">
         <is>
           <t>c7989fc1-f256-4159-9c4c-ae3f481836ff</t>
@@ -2996,6 +3001,11 @@
           <t>Float</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>K.O.</t>
@@ -3021,6 +3031,11 @@
       </c>
       <c r="N8" t="n">
         <v>15</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Minimum Coefficient of Performance required — ratio of refrigeration output to electrical power input (e.g. COP 3.5 means 3.5 kW cooling per 1 kW electricity)</t>
+        </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -6135,8 +6150,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
OI-85: Fix classification guide double-arrow bug in AP0 + generate_all.py
Root cause: AGV leaf nodes in AP0 ③ Scope Registry had classification_guide
cells starting with * "alias" →; generate_all.py prepended * "canonical" →,
creating double-arrows like * "Forklift AGV" → * "VNA" → in all classification
and extraction templates.

Fix: re-author 3 AP0 cells to plain canonical descriptions + populate
variant_guide_json for Forklift (5 sub-variants) and AMR (Underride AMR);
centralize 3 render sites in generate_all.py into _render_leaf_scope_lines()
helper that outputs sub-variants as indented bullets. FoodBev:Refrigeration
unaffected (uses dom_variant_guides path). 248 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -5028,11 +5028,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>* "VNA" → AGV stores/retrieves in very narrow aisles (&lt;2m), lifts to tall racking (&gt;8m), high-bay warehouse. ONLY classify as VNA if the tender explicitly requires VNA capability for the AGVs being procured. If VNA racking is mentioned as existing infrastructure, historical context, or out-of-scope aisles not covered by this tender — do NOT classify as VNA. Signals: aisle&lt;2m, lift&gt;8m, high-bay, VNA keyword
-* "Very Narrow Aisle" → Same as VNA
-* "Reach Truck" → AGV picks/places in medium-width racking aisles (2–3m), lift 4–8m. Signals: 2–3m aisle, racking, lift 4–8m
-* "Counterbalanced" → AGV transports pallets on wide aisles (≥3m) or open floor between fixed transfer stations, floor-level pickup/deposit. USE THIS for heavy pallet transport (&gt;1000 kg) in F&amp;B, food production, or manufacturing environments — even when MES or OPC-UA integration is mentioned. The presence of filling lines or MES does NOT imply Mobile AMR if payload is heavy. Signals: ≥3m aisle, floor transport, transfer stations, warehouse/logistics, heavy pallet (&gt;1000 kg)
-* "Forklift" → Generic forklift AGV</t>
+          <t>Pallet-lifting fork-based AGV for transport, picking, and placing of pallets, IBCs, and similar loads.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -5063,6 +5059,11 @@
           <t>VNA (very narrow aisle) operation is required.</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>{"VNA": "AGV stores/retrieves in very narrow aisles (&lt;2m), lifts to tall racking (&gt;8m), high-bay warehouse. ONLY classify as VNA if the tender explicitly requires VNA capability for the AGVs being procured. If VNA racking is mentioned as existing infrastructure, historical context, or out-of-scope aisles not covered by this tender — do NOT classify as VNA. Signals: aisle&lt;2m, lift&gt;8m, high-bay, VNA keyword", "Very Narrow Aisle": "Same as VNA", "Reach Truck": "AGV picks/places in medium-width racking aisles (2–3m), lift 4–8m. Signals: 2–3m aisle, racking, lift 4–8m", "Counterbalanced": "AGV transports pallets on wide aisles (≥3m) or open floor between fixed transfer stations, floor-level pickup/deposit. USE THIS for heavy pallet transport (&gt;1000 kg) in F&amp;B, food production, or manufacturing environments — even when MES or OPC-UA integration is mentioned. The presence of filling lines or MES does NOT imply Mobile AMR if payload is heavy. Signals: ≥3m aisle, floor transport, transfer stations, warehouse/logistics, heavy pallet (&gt;1000 kg)", "Forklift": "Generic forklift AGV"}</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5092,7 +5093,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>* "Tugger" → AGV tows a train of trolleys/trailers without lifting; no direct pallet fork interface. Signals: trailer train, towing, milk run</t>
+          <t>AGV tows a train of trolleys/trailers without lifting; no direct pallet fork interface. Signals: trailer train, towing, milk run</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -5144,8 +5145,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>* "Mobile AMR" → Autonomous robot in PRODUCTION or MANUFACTURING environment (filling lines, assembly, processing), or with conveyor/shelf top modules, SLAM navigation, dispatched from MES/WMS. ONLY use for LIGHT payloads (typically &lt;1000 kg). If payload &gt;1000 kg or if the task is heavy pallet transport → use Forklift AGV instead. Signals: production, filling lines, manufacturing, SLAM, MES — BUT only if payload &lt;1000 kg
-* "Underride AMR" → Robot slides under carts/dollies and lifts them a few cm for transport. Signals: underride, dolly, cart</t>
+          <t>Autonomous robot in PRODUCTION or MANUFACTURING environment (filling lines, assembly, processing), or with conveyor/shelf top modules, SLAM navigation, dispatched from MES/WMS. ONLY use for LIGHT payloads (typically &lt;1000 kg). If payload &gt;1000 kg or if the task is heavy pallet transport → use Forklift AGV instead. Signals: production, filling lines, manufacturing, SLAM, MES — BUT only if payload &lt;1000 kg</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -5166,6 +5166,11 @@
       <c r="M6" t="inlineStr">
         <is>
           <t>amr_specific</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>{"Underride AMR": "Robot slides under carts/dollies and lifts them a few cm for transport. Signals: underride, dolly, cart"}</t>
         </is>
       </c>
     </row>
@@ -6150,9 +6155,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
OI-88: Strip alias prefix from FoodBev:Refrigeration classification_guide
Same root cause as OI-85: FoodBev classification_guide cell started with
* "Industrial Refrigeration" → (alias format), producing a double-arrow in
combined fallback templates. Fixed by stripping the prefix — now a plain
canonical description, consistent with the invariant established in OI-85.

Combined templates (scope_classification_template.txt, vehicle_type_template.txt,
extraction_template.txt) are now clean across all domains. 248 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>* "Industrial Refrigeration" → Industrial refrigeration system for food &amp; beverage: process cooling, cold storage, or deep-freeze applications. Keywords: Kälteanlage, Kältetechnik, refrigeration, industrial cooling, cold store, deep freeze, blast freezer.</t>
+          <t>Industrial refrigeration system for food &amp; beverage: process cooling, cold storage, or deep-freeze applications. Keywords: Kälteanlage, Kältetechnik, refrigeration, industrial cooling, cold store, deep freeze, blast freezer.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -6155,9 +6155,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B5:F5"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
OI-84/86: Add VNA golden assertion + fix max_gradient_pct AP0 hint
OI-84: tender_005.json golden_extraction now asserts required_vna_capable="not_required"
and required_product_type="Forklift AGV" — closes the KO_BOOL_EXCLUSIVE regression blind
spot where a VNA false-positive would silently eliminate nearly all supplier matches.

OI-86: AP0 LLM Hint for max_gradient_pct (AGV_Shared) revised — removed the biasing
"most flat indoor warehouse floors have 0% gradient" phrase and numeric literals (10%/5.7°).
Added explicit rule: approximate values ("approximately X%") count as explicit and must not
be nulled. Addresses non-deterministic extraction of the genuine CompanyX 1.5% gradient.

248 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -6155,8 +6155,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B3:F3"/>
     <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7089,7 +7089,7 @@
       </c>
       <c r="G22" s="68" t="inlineStr">
         <is>
-          <t>Max ramp gradient the loaded unit handles. Source: spec 'gradeability' — must appear as an explicit % value. The value represents the steepest ramp gradient (%) the loaded vehicle must climb: 10 % ≈ 5.7° incline; most flat indoor warehouse floors have 0 % gradient and this field should be null. Cond. K.O.: binds only where the site has ramps/dock inclines. NULL RULE: null unless a slope or gradient percentage is explicitly stated in the document. Do NOT apply typical industry values (e.g. '5%') when the document is silent on gradients.</t>
+          <t>Max ramp gradient the loaded unit handles. Source: spec 'gradeability' — must appear as an explicit % value. The value represents the steepest ramp gradient (%) the loaded vehicle must climb. Cond. K.O.: binds only where the site has ramps/dock inclines. NULL RULE: null unless a slope or gradient percentage is explicitly stated in the document. An approximate value (e.g. 'approximately X%') counts as explicit — do not null it solely because the document qualifies the figure. Do NOT infer or apply typical values when the document is silent on gradients.</t>
         </is>
       </c>
       <c r="H22" s="52" t="inlineStr">

</xml_diff>

<commit_message>
Fix shared-scope dialog bug + remove load_type "None" from AP0
Dialog scope fix (sharedScope regression from OI-81 refactor):
_fieldMeta.__vt_config__.shared_scope was removed during OI-81 but the
frontend still read it, defaulting to '' — silently excluding all
AGV_Shared fields (max_payload_kg, load_type, etc.) from both the
Clarification and Edit dialogs. Fixed in buildClarificationFields,
buildEditFields, buildAddFieldPicker by deriving sharedScope from the
domains array already present in __vt_config__.

load_type "None" removed from AP0 allowed_values:
"None" in a KO_SUBSET AND field would KO every supplier (no supplier
has load_type=None). It was a UI placeholder, not a real matchable
value. Blank selection in the dialog already maps to null via LL-06,
so no functional change — just removes the trap.

248 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -6155,9 +6155,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -6594,7 +6594,7 @@
       </c>
       <c r="C11" s="69" t="inlineStr">
         <is>
-          <t>None | Pallet EUR | Pallet ISO | Half-Euro | UK Pallet | Medium Euro | Tote | Plastic Bin | Bulk Bin | Roll Container | Custom Carrier</t>
+          <t>Pallet EUR | Pallet ISO | Half-Euro | UK Pallet | Medium Euro | Tote | Plastic Bin | Bulk Bin | Roll Container | Custom Carrier</t>
         </is>
       </c>
       <c r="E11" s="25" t="inlineStr">

</xml_diff>

<commit_message>
OI-89 + OI-92: Fix replay detected_domain + cop_efficiency KO→SCORING
OI-89: Replay path (app.py) failed to set detected_domain for old JSON
captures that pre-date the field — showResult() hid agvSection entirely.
Fix: derive detected_domain from VT's leaf scope via LEGACY_MAP +
_EXTRACTABLE_DOMAINS when not present in cached JSON.

OI-92: cop_efficiency was misconfigured as K.O./KO_IF_LT in AP0
FoodBev_Refrigeration — caused it to wrongly appear in Clarification
Dialog and disqualify suppliers. Corrected to Scoring/no operator.

248 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -3008,7 +3008,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>K.O.</t>
+          <t>Scoring</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3019,11 +3019,6 @@
       <c r="G8" t="inlineStr">
         <is>
           <t>Extract the COP (Coefficient of Performance) at rated conditions. Use the highest stated COP. NULL RULE: return null if not stated.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>KO_IF_LT</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -6155,9 +6150,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
OI-92 (amend): cop_efficiency → Cond. K.O. / KO_IF_LT
Corrects the previous commit which set it to Scoring.
Original KO intent (IK Sprint Phase 3) was deliberate — hard COP floor
for refrigeration tenders. COND_KO is the right level (conditional on
whether tender specifies a COP requirement). 248 tests green.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -3008,7 +3008,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Scoring</t>
+          <t>Cond. K.O.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3019,6 +3019,11 @@
       <c r="G8" t="inlineStr">
         <is>
           <t>Extract the COP (Coefficient of Performance) at rated conditions. Use the highest stated COP. NULL RULE: return null if not stated.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>KO_IF_LT</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -6150,9 +6155,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
OI-103: Remove VNA derivation machinery — LLM extracts vna_capable as regular 4b field
- Remove _VNA_CFG, _VNA_APPLICABLE, _VNA_CONTEXT_HINT startup constants (app.py)
- Remove is_vna_subtype variable, vna_label, vna_context, all related branches (app.py)
- Remove 4a→4b vna_capable merge, rematch special-case, result["is_vna"] (app.py)
- Remove outdoor_capable normalization block — covered by Option B (_op_bool_exclusive)
- _AP0_SKIP_VALIDATION now empty frozenset; _SKIP_FILTER only {"required_product_type"}
- _op_bool_exclusive: accept boolean true/yes/false/no from LLM output (matching.py)
- Remove required_vna_capable from _4A_FIELDS; remove {vna_context} placeholder (generate_all.py)
- Remove vna_capable from 4a template JSON schema + guidance text (generate_all.py)
- AP0: revised vna_capable hint (explicit VNA mandate only, default=false), vna_subtypes cleared
- 248 tests green; all DoD checks passed

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -2149,7 +2149,7 @@
       </c>
       <c r="C3" s="54" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D3" s="54" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="C4" s="54" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D4" s="54" t="inlineStr">
@@ -6155,9 +6155,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B5:F5"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="G10" s="68" t="inlineStr">
         <is>
-          <t>VNA / very narrow aisle operation required. true/false. Source: 'VNA', aisle &lt; 2 m with high-bay racking. If true, required_drive_type must be 'VNA Turret'.</t>
+          <t>Set to true ONLY if this tender explicitly mandates VNA (Very Narrow Aisle) capability — aisle widths below 1.8 m requiring turret or side-loader technology. Set to false if VNA is not mentioned or standard aisles are assumed — this is the default for standard Forklift AGV tenders. Do NOT set to true if VNA is mentioned only as existing warehouse context, historical infrastructure, or areas outside this procurement scope. Null only if aisle requirements are genuinely ambiguous.</t>
         </is>
       </c>
       <c r="H10" s="52" t="inlineStr">

</xml_diff>

<commit_message>
IK Sprint Phase 6: SA-23 country ISO-format hint (AP0 + fields.json)
SA pre-plan check found the originally planned allowed_values fix would
be a no-op (full ISO catalog) or actively harmful (curated list nulls
legitimate values / lets wrong-vocabulary values through, disqualifying
suppliers via KO_SUBSET). required_country has a clean 33/33 null
record with zero observed hallucinations, so the effective fix is a
single AP0 Description cell addition instructing ISO 3166-1 alpha-2
output — no example codes, to avoid prompt-poisoning a field with a
clean record. allowed_values/data_type left untouched.

302 tests green; historical corpus replay confirms required_country
stays null.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -905,7 +905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>HQ country of the selling company. Used as Cond. K.O. when buyer requires domestic or regional supplier. NULL RULE: output null unless the tender explicitly requires a domestic or specific-country supplier. Do NOT infer from buyer address or document language.</t>
+          <t>HQ country of the selling company. Used as Cond. K.O. when buyer requires domestic or regional supplier. NULL RULE: output null unless the tender explicitly requires a domestic or specific-country supplier. Do NOT infer from buyer address or document language. If a country requirement is stated, output the 2-letter ISO 3166-1 alpha-2 code in uppercase. Never output a country name, a region, or a word meaning "domestic".</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -6175,9 +6175,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B5:F5"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
IK Sprint Phase 8: Hygiene-Bündel (D5+D6+D8+OI-72)
- D6: remove duplicated CONSERVATIVE EXTRACTION sentence from max_payload_kg's
  AP0 hint (generate_all.py auto-appends it already); new generation-time
  guardrail asserts no future field can reintroduce this collision.
- D8: haystacked.log now rotates (RotatingFileHandler, 20MB x 5 backups)
  instead of growing unbounded; prior 270MB log archived under docs/archive/.
- D5: replace stale hardcoded _FIXED_OVERHEAD_TOKENS (10,100) with a dynamic
  calculation from the actual system-prompt + 4b-template lengths.
- OI-72: verified end-to-end via /analyze + /rematch that a gradient
  requirement of 0 is correctly treated as "no constraint" (src/matching.py
  KO_IF_LT zero-exemption), not a hard KO.

Reviewed by senior-architect, ap0-architecture-guardian, and
reference-integrity-guardian before implementation. 313 tests green.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Spec/haystacked_AP0_field_spec_v0_10.xlsx
+++ b/Spec/haystacked_AP0_field_spec_v0_10.xlsx
@@ -6170,9 +6170,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -6576,7 +6576,7 @@
       </c>
       <c r="G10" s="68" t="inlineStr">
         <is>
-          <t>Maximum payload the AGV must carry per trip, in kg. This value may appear as prose (e.g. 'a maximum of X kg', 'loads up to X kg', 'pallets weigh up to X kg') OR as a table column (labelled 'Max Loaded weight' / 'gross weight'). Read BOTH prose sentences and table cells — do not restrict search to tables only. In tables, use the loaded/gross weight — IGNORE 'tare weight' / 'empty pallet weight'. If a range or several load types are given, report the heaviest stated number. NULL RULE: Output null only if no maximum load weight is stated anywhere in the document text. CONSERVATIVE EXTRACTION: if multiple values are stated, extract the MAXIMUM — the supplier must meet or exceed this threshold.</t>
+          <t>Maximum payload the AGV must carry per trip, in kg. This value may appear as prose (e.g. 'a maximum of X kg', 'loads up to X kg', 'pallets weigh up to X kg') OR as a table column (labelled 'Max Loaded weight' / 'gross weight'). Read BOTH prose sentences and table cells — do not restrict search to tables only. In tables, use the loaded/gross weight — IGNORE 'tare weight' / 'empty pallet weight'. If a range or several load types are given, report the heaviest stated number. NULL RULE: Output null only if no maximum load weight is stated anywhere in the document text.</t>
         </is>
       </c>
       <c r="H10" s="52" t="inlineStr">

</xml_diff>